<commit_message>
Fix version label from 'snapsnot' to 'snapshot' (#115) eae606c39069f621b4f7f18ef796f1c6bf3833c1
</commit_message>
<xml_diff>
--- a/main/ig/FRActSubstitutionLMCDAFHIR.xlsx
+++ b/main/ig/FRActSubstitutionLMCDAFHIR.xlsx
@@ -31,7 +31,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0-snapsnot</t>
+    <t>0.1.0-snapshot</t>
   </si>
   <si>
     <t>Name</t>
@@ -55,7 +55,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-07T08:23:13+00:00</t>
+    <t>2026-04-15T13:29:57+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>